<commit_message>
Standaizd the packing slips, added a "raw" inventory upload feature, added a basic network provisioning and validated working on 7705/7250 with quarks, added support for SAOS 6 + 10 but are untested, refactored from single thread to multi thread and reduced the amout of logins per device to 1
</commit_message>
<xml_diff>
--- a/data/Device_Report_Template.xlsx
+++ b/data/Device_Report_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lightriver-my.sharepoint.com/personal/zsimino_lightriver_com/Documents/Documents/Programs/network_inventory/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZackerySimino\Downloads\LAMIS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="359" documentId="8_{9CB5FA86-B0E6-4949-A545-39C05F0C244E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC6245D0-E2A4-4598-9F4D-AF946B0E0DE5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E510856-E3CD-4C55-A263-D7F107445C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1CE12A3A-5550-47E4-8A53-A8AE70C33086}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{1CE12A3A-5550-47E4-8A53-A8AE70C33086}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer-project" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Customer:</t>
   </si>
@@ -82,12 +82,15 @@
   <si>
     <t>Customer PO/Sale Order:</t>
   </si>
+  <si>
+    <t>Asset Tag</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,6 +150,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -168,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -192,19 +202,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -318,39 +315,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -370,45 +334,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -466,21 +391,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -501,6 +411,41 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -508,9 +453,31 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -518,15 +485,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -538,106 +505,106 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1023,119 +990,131 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88A4540E-060F-4722-81FE-D7263FE19264}">
-  <dimension ref="B1:F93"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B1:G93"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="5" width="27.08984375" customWidth="1"/>
-    <col min="6" max="6" width="40.81640625" customWidth="1"/>
-    <col min="7" max="7" width="23.54296875" customWidth="1"/>
+    <col min="2" max="5" width="27.140625" customWidth="1"/>
+    <col min="6" max="6" width="40.85546875" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="27" t="s">
+    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="29"/>
-    </row>
-    <row r="3" spans="2:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="32"/>
-    </row>
-    <row r="4" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="19"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="20"/>
+    </row>
+    <row r="4" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="21"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="20"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="26"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="20"/>
-    </row>
-    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F5" s="27"/>
+      <c r="G5" s="29"/>
+    </row>
+    <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="47"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
       <c r="E6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="21"/>
-    </row>
-    <row r="7" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="10" t="s">
+      <c r="F6" s="28"/>
+      <c r="G6" s="30"/>
+    </row>
+    <row r="7" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="11" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="22"/>
-    </row>
-    <row r="8" spans="2:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="39"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="41"/>
-    </row>
-    <row r="9" spans="2:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="42"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="44"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="36" t="s">
+      <c r="F7" s="35"/>
+      <c r="G7" s="30"/>
+    </row>
+    <row r="8" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="36"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="38"/>
+    </row>
+    <row r="9" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="23"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="25"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="17"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="14"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="36" t="s">
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="38"/>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="12" t="s">
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="10" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1144,560 +1123,641 @@
       <c r="D14" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="10" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G14" s="42" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G16" s="13"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G20" s="13"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G21" s="13"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="13"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24"/>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="24"/>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="24"/>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="24"/>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E47" s="13"/>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="24"/>
-      <c r="F49" s="24"/>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="24"/>
-      <c r="F50" s="24"/>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
-      <c r="E52" s="24"/>
-      <c r="F52" s="24"/>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E52" s="13"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="24"/>
-      <c r="F53" s="24"/>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="24"/>
-      <c r="F54" s="24"/>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
-    </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E56" s="13"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="24"/>
-      <c r="F57" s="24"/>
-    </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-    </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="G59" s="13"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="24"/>
-      <c r="F60" s="24"/>
-    </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E60" s="13"/>
+      <c r="F60" s="13"/>
+      <c r="G60" s="13"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="24"/>
-      <c r="F61" s="24"/>
-    </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="G61" s="13"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="24"/>
-      <c r="F62" s="24"/>
-    </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E62" s="13"/>
+      <c r="F62" s="13"/>
+      <c r="G62" s="13"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-    </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E63" s="13"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="13"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-    </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E64" s="13"/>
+      <c r="F64" s="13"/>
+      <c r="G64" s="13"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
-    </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E65" s="13"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="13"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="24"/>
-    </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E66" s="13"/>
+      <c r="F66" s="13"/>
+      <c r="G66" s="13"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-    </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="24"/>
-      <c r="F68" s="24"/>
-    </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E68" s="13"/>
+      <c r="F68" s="13"/>
+      <c r="G68" s="13"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="24"/>
-      <c r="F69" s="24"/>
-    </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E69" s="13"/>
+      <c r="F69" s="13"/>
+      <c r="G69" s="13"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="24"/>
-      <c r="F70" s="24"/>
-    </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E70" s="13"/>
+      <c r="F70" s="13"/>
+      <c r="G70" s="13"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="24"/>
-      <c r="F71" s="24"/>
-    </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E71" s="13"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="13"/>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
-      <c r="E72" s="24"/>
-      <c r="F72" s="24"/>
-    </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E72" s="13"/>
+      <c r="F72" s="13"/>
+      <c r="G72" s="13"/>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
-      <c r="E73" s="24"/>
-      <c r="F73" s="24"/>
-    </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E73" s="13"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="13"/>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
-      <c r="E74" s="24"/>
-      <c r="F74" s="24"/>
-    </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E74" s="13"/>
+      <c r="F74" s="13"/>
+      <c r="G74" s="13"/>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
       <c r="D75" s="4"/>
-      <c r="E75" s="24"/>
-      <c r="F75" s="24"/>
-    </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B76" s="23"/>
+      <c r="E75" s="13"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="13"/>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B76" s="12"/>
       <c r="C76" s="4"/>
       <c r="D76" s="5"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="24"/>
-    </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B77" s="23"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
+      <c r="G76" s="13"/>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B77" s="12"/>
       <c r="C77" s="4"/>
       <c r="D77" s="5"/>
-      <c r="E77" s="24"/>
-      <c r="F77" s="24"/>
-    </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B78" s="23"/>
+      <c r="E77" s="13"/>
+      <c r="F77" s="13"/>
+      <c r="G77" s="13"/>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="12"/>
       <c r="C78" s="4"/>
       <c r="D78" s="5"/>
-      <c r="E78" s="24"/>
-      <c r="F78" s="24"/>
-    </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B79" s="23"/>
+      <c r="E78" s="13"/>
+      <c r="F78" s="13"/>
+      <c r="G78" s="13"/>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B79" s="12"/>
       <c r="C79" s="4"/>
       <c r="D79" s="5"/>
-      <c r="E79" s="24"/>
-      <c r="F79" s="24"/>
-    </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B80" s="23"/>
+      <c r="E79" s="13"/>
+      <c r="F79" s="13"/>
+      <c r="G79" s="13"/>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B80" s="12"/>
       <c r="C80" s="4"/>
       <c r="D80" s="5"/>
-      <c r="E80" s="24"/>
-      <c r="F80" s="24"/>
-    </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B81" s="23"/>
+      <c r="E80" s="13"/>
+      <c r="F80" s="13"/>
+      <c r="G80" s="13"/>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B81" s="12"/>
       <c r="C81" s="4"/>
       <c r="D81" s="5"/>
-      <c r="E81" s="24"/>
-      <c r="F81" s="24"/>
-    </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B82" s="23"/>
+      <c r="E81" s="13"/>
+      <c r="F81" s="13"/>
+      <c r="G81" s="13"/>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B82" s="12"/>
       <c r="C82" s="4"/>
       <c r="D82" s="5"/>
-      <c r="E82" s="24"/>
-      <c r="F82" s="24"/>
-    </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B83" s="23"/>
+      <c r="E82" s="13"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="13"/>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B83" s="12"/>
       <c r="C83" s="4"/>
       <c r="D83" s="5"/>
-      <c r="E83" s="24"/>
-      <c r="F83" s="24"/>
-    </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B84" s="23"/>
+      <c r="E83" s="13"/>
+      <c r="F83" s="13"/>
+      <c r="G83" s="13"/>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B84" s="12"/>
       <c r="C84" s="4"/>
       <c r="D84" s="5"/>
-      <c r="E84" s="24"/>
-      <c r="F84" s="24"/>
-    </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B85" s="23"/>
+      <c r="E84" s="13"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="13"/>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B85" s="12"/>
       <c r="C85" s="4"/>
       <c r="D85" s="5"/>
-      <c r="E85" s="24"/>
-      <c r="F85" s="24"/>
-    </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B86" s="23"/>
+      <c r="E85" s="13"/>
+      <c r="F85" s="13"/>
+      <c r="G85" s="13"/>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B86" s="12"/>
       <c r="C86" s="4"/>
       <c r="D86" s="5"/>
-      <c r="E86" s="24"/>
-      <c r="F86" s="24"/>
-    </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B87" s="23"/>
+      <c r="E86" s="13"/>
+      <c r="F86" s="13"/>
+      <c r="G86" s="13"/>
+    </row>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B87" s="12"/>
       <c r="C87" s="4"/>
       <c r="D87" s="5"/>
-      <c r="E87" s="24"/>
-      <c r="F87" s="24"/>
-    </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B88" s="23"/>
+      <c r="E87" s="13"/>
+      <c r="F87" s="13"/>
+      <c r="G87" s="13"/>
+    </row>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B88" s="12"/>
       <c r="C88" s="4"/>
       <c r="D88" s="5"/>
-      <c r="E88" s="24"/>
-      <c r="F88" s="24"/>
-    </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E88" s="13"/>
+      <c r="F88" s="13"/>
+      <c r="G88" s="13"/>
+    </row>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
       <c r="D89" s="5"/>
-      <c r="E89" s="24"/>
-      <c r="F89" s="24"/>
-    </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E89" s="13"/>
+      <c r="F89" s="13"/>
+      <c r="G89" s="13"/>
+    </row>
+    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
       <c r="D90" s="5"/>
-      <c r="E90" s="24"/>
-      <c r="F90" s="24"/>
-    </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E90" s="13"/>
+      <c r="F90" s="13"/>
+      <c r="G90" s="13"/>
+    </row>
+    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
       <c r="D91" s="5"/>
-      <c r="E91" s="24"/>
-      <c r="F91" s="24"/>
-    </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E91" s="13"/>
+      <c r="F91" s="13"/>
+      <c r="G91" s="13"/>
+    </row>
+    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
       <c r="D92" s="5"/>
-      <c r="E92" s="24"/>
-      <c r="F92" s="24"/>
-    </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E92" s="13"/>
+      <c r="F92" s="13"/>
+      <c r="G92" s="13"/>
+    </row>
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
       <c r="D93" s="1"/>
@@ -1707,11 +1767,14 @@
       <c r="F93" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B2:F4"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B8:F9"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:G4"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="B8:G9"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>